<commit_message>
Tweaks to figure and data file
</commit_message>
<xml_diff>
--- a/data/lab_personnel_timeline.xlsx
+++ b/data/lab_personnel_timeline.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Utku\Lab_personnel_timeline\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ken\github\campbellmusclelab\lab\Lab_personnel_timeline\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADBB3334-5A02-4DBE-A93F-178A8E301333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBEB92BF-C90E-4D83-9775-3F7081F8D6A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="32520" windowHeight="15495" xr2:uid="{894F3479-6172-4C97-B34D-DB9478A5D1D4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{894F3479-6172-4C97-B34D-DB9478A5D1D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -77,9 +77,6 @@
     <t>Minton</t>
   </si>
   <si>
-    <t>Rotation mentor</t>
-  </si>
-  <si>
     <t>Mason</t>
   </si>
   <si>
@@ -95,9 +92,6 @@
     <t>Tinnell</t>
   </si>
   <si>
-    <t>Medical students</t>
-  </si>
-  <si>
     <t>Chandler</t>
   </si>
   <si>
@@ -633,6 +627,12 @@
   </si>
   <si>
     <t>Mallamaci</t>
+  </si>
+  <si>
+    <t>Medical student</t>
+  </si>
+  <si>
+    <t>Rotation mentee</t>
   </si>
 </sst>
 </file>
@@ -1067,7 +1067,7 @@
         <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D4" s="2">
         <v>45139</v>
@@ -1078,13 +1078,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D5" s="2">
         <v>44927</v>
@@ -1095,13 +1095,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="B6" t="s">
-        <v>18</v>
-      </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>197</v>
       </c>
       <c r="D6" s="2">
         <v>45078</v>
@@ -1112,13 +1112,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
         <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" t="s">
-        <v>22</v>
       </c>
       <c r="D7" s="1">
         <v>44044</v>
@@ -1129,13 +1129,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D8" s="2">
         <v>43678</v>
@@ -1146,13 +1146,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
         <v>25</v>
-      </c>
-      <c r="B9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" t="s">
-        <v>27</v>
       </c>
       <c r="D9" s="2">
         <v>44044</v>
@@ -1163,13 +1163,13 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D10" s="2">
         <v>43313</v>
@@ -1183,10 +1183,10 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D11" s="2">
         <v>44105</v>
@@ -1197,13 +1197,13 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D12" s="2">
         <v>43678</v>
@@ -1214,13 +1214,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D13" s="2">
         <v>43678</v>
@@ -1248,13 +1248,13 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D15" s="2">
         <v>42948</v>
@@ -1265,13 +1265,13 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D16" s="2">
         <v>43313</v>
@@ -1282,13 +1282,13 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D17" s="2">
         <v>43313</v>
@@ -1299,13 +1299,13 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" t="s">
         <v>40</v>
-      </c>
-      <c r="B18" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" t="s">
-        <v>42</v>
       </c>
       <c r="D18" s="2">
         <v>43101</v>
@@ -1316,13 +1316,13 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D19" s="2">
         <v>42948</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C20" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D20" s="1">
         <v>41487</v>
@@ -1350,13 +1350,13 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D21" s="2">
         <v>42217</v>
@@ -1367,13 +1367,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D22" s="2">
         <v>42217</v>
@@ -1384,13 +1384,13 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" t="s">
         <v>51</v>
-      </c>
-      <c r="B23" t="s">
-        <v>52</v>
-      </c>
-      <c r="C23" t="s">
-        <v>53</v>
       </c>
       <c r="D23" s="2">
         <v>41487</v>
@@ -1401,13 +1401,13 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D24" s="2">
         <v>42583</v>
@@ -1418,13 +1418,13 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C25" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D25" s="2">
         <v>42217</v>
@@ -1435,13 +1435,13 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C26" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D26" s="2">
         <v>42217</v>
@@ -1452,13 +1452,13 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B27" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C27" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D27" s="2">
         <v>42005</v>
@@ -1469,13 +1469,13 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B28" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C28" t="s">
-        <v>19</v>
+        <v>197</v>
       </c>
       <c r="D28" s="2">
         <v>42005</v>
@@ -1486,13 +1486,13 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B29" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C29" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D29" s="2">
         <v>41852</v>
@@ -1503,13 +1503,13 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B30" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C30" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D30" s="2">
         <v>41122</v>
@@ -1520,13 +1520,13 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B31" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C31" t="s">
-        <v>19</v>
+        <v>197</v>
       </c>
       <c r="D31" s="2">
         <v>41640</v>
@@ -1537,13 +1537,13 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C32" t="s">
-        <v>19</v>
+        <v>197</v>
       </c>
       <c r="D32" s="2">
         <v>41640</v>
@@ -1554,13 +1554,13 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B33" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C33" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D33" s="2">
         <v>41852</v>
@@ -1571,13 +1571,13 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C34" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D34" s="2">
         <v>41852</v>
@@ -1588,13 +1588,13 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B35" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C35" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D35" s="2">
         <v>41640</v>
@@ -1605,13 +1605,13 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B36" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C36" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D36" s="2">
         <v>41122</v>
@@ -1622,13 +1622,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B37" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C37" t="s">
-        <v>19</v>
+        <v>197</v>
       </c>
       <c r="D37" s="2">
         <v>41487</v>
@@ -1639,13 +1639,13 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C38" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D38" s="2">
         <v>40026</v>
@@ -1656,13 +1656,13 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B39" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C39" t="s">
-        <v>19</v>
+        <v>197</v>
       </c>
       <c r="D39" s="2">
         <v>41275</v>
@@ -1673,13 +1673,13 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B40" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C40" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D40" s="2">
         <v>41122</v>
@@ -1690,13 +1690,13 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C41" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D41" s="2">
         <v>41122</v>
@@ -1707,13 +1707,13 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B42" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C42" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D42" s="2">
         <v>41275</v>
@@ -1724,13 +1724,13 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B43" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C43" t="s">
-        <v>19</v>
+        <v>197</v>
       </c>
       <c r="D43" s="2">
         <v>41122</v>
@@ -1741,13 +1741,13 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B44" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C44" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D44" s="2">
         <v>41122</v>
@@ -1758,13 +1758,13 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B45" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C45" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D45" s="2">
         <v>40391</v>
@@ -1775,13 +1775,13 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B46" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C46" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D46" s="2">
         <v>40756</v>
@@ -1792,10 +1792,10 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B47" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C47" t="s">
         <v>7</v>
@@ -1809,13 +1809,13 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B48" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C48" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D48" s="1">
         <v>40391</v>
@@ -1826,13 +1826,13 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B49" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C49" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D49" s="2">
         <v>40560</v>
@@ -1843,13 +1843,13 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B50" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C50" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D50" s="2">
         <v>40560</v>
@@ -1860,13 +1860,13 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B51" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C51" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D51" s="2">
         <v>39295</v>
@@ -1877,13 +1877,13 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B52" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C52" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D52" s="1">
         <v>40391</v>
@@ -1894,13 +1894,13 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B53" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C53" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D53" s="1">
         <v>40391</v>
@@ -1911,13 +1911,13 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B54" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C54" t="s">
-        <v>19</v>
+        <v>197</v>
       </c>
       <c r="D54" s="2">
         <v>39965</v>
@@ -1928,13 +1928,13 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B55" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C55" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D55" s="1">
         <v>39661</v>
@@ -1945,10 +1945,10 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B56" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C56" t="s">
         <v>7</v>
@@ -1962,13 +1962,13 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B57" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C57" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D57" s="2">
         <v>39661</v>
@@ -1979,13 +1979,13 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B58" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C58" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D58" s="2">
         <v>39661</v>
@@ -1996,13 +1996,13 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B59" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C59" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D59" s="1">
         <v>39295</v>
@@ -2013,13 +2013,13 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B60" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C60" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D60" s="1">
         <v>39295</v>
@@ -2030,13 +2030,13 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B61" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C61" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D61" s="2">
         <v>39295</v>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B62" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C62" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D62" s="1">
         <v>38930</v>
@@ -2067,10 +2067,10 @@
         <v>5</v>
       </c>
       <c r="B63" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C63" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D63" s="1">
         <v>38930</v>
@@ -2081,13 +2081,13 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B64" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D64" s="2">
         <v>38930</v>
@@ -2098,13 +2098,13 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B65" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C65" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D65" s="2">
         <v>38930</v>
@@ -2115,13 +2115,13 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B66" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C66" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D66" s="2">
         <v>38930</v>
@@ -2132,13 +2132,13 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B67" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C67" t="s">
-        <v>13</v>
+        <v>198</v>
       </c>
       <c r="D67" s="2">
         <v>38200</v>
@@ -2149,13 +2149,13 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B68" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C68" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D68" s="1">
         <v>38169</v>
@@ -2163,10 +2163,10 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B69" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C69" t="s">
         <v>7</v>
@@ -2180,13 +2180,13 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B70" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C70" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D70" s="1">
         <v>44562</v>
@@ -2197,13 +2197,13 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B71" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C71" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D71" s="1">
         <v>45161</v>
@@ -2212,13 +2212,13 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B72" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C72" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D72" s="1">
         <v>45139</v>
@@ -2226,13 +2226,13 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B73" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C73" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D73" s="1">
         <v>45444</v>
@@ -2243,13 +2243,13 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B74" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C74" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D74" s="2">
         <v>45170</v>
@@ -2260,13 +2260,13 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B75" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C75" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D75" s="2">
         <v>45292</v>
@@ -2277,13 +2277,13 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B76" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C76" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D76" s="2">
         <v>45170</v>
@@ -2294,13 +2294,13 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B77" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C77" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D77" s="2">
         <v>45383</v>
@@ -2311,13 +2311,13 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B78" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C78" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D78" s="2">
         <v>45383</v>
@@ -2328,13 +2328,13 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B79" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C79" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D79" s="2">
         <v>45383</v>
@@ -2343,13 +2343,13 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B80" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C80" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D80" s="2">
         <v>44409</v>
@@ -2363,16 +2363,16 @@
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C81" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D81" s="2">
         <v>44409</v>
       </c>
       <c r="E81" s="2">
-        <v>46381</v>
+        <v>46016</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
@@ -2383,7 +2383,7 @@
         <v>12</v>
       </c>
       <c r="C82" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D82" s="2">
         <v>45139</v>
@@ -2392,13 +2392,13 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B83" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C83" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D83" s="2">
         <v>45505</v>
@@ -2407,13 +2407,13 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B84" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C84" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D84" s="2">
         <v>44774</v>
@@ -2424,13 +2424,13 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B85" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C85" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D85" s="2">
         <v>45536</v>
@@ -2439,13 +2439,13 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B86" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C86" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D86" s="2">
         <v>45139</v>
@@ -2454,13 +2454,13 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B87" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C87" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D87" s="2">
         <v>45505</v>
@@ -2471,13 +2471,13 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B88" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D88" s="2">
         <v>42401</v>
@@ -2488,13 +2488,13 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B89" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C89" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D89" s="1">
         <v>45292</v>
@@ -2502,13 +2502,13 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B90" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C90" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D90" s="1">
         <v>45566</v>
@@ -2516,13 +2516,13 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B91" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C91" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D91" s="1">
         <v>45658</v>
@@ -2530,13 +2530,13 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B92" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C92" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D92" s="1">
         <v>45658</v>
@@ -2544,13 +2544,13 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B93" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C93" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D93" s="1">
         <v>45658</v>
@@ -2558,13 +2558,13 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B94" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C94" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D94" s="1">
         <v>45658</v>
@@ -2572,13 +2572,13 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B95" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C95" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D95" s="1">
         <v>45597</v>
@@ -2589,13 +2589,13 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B96" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C96" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D96" s="1">
         <v>45658</v>
@@ -2603,13 +2603,13 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B97" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C97" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D97" s="1">
         <v>45658</v>
@@ -2617,13 +2617,13 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B98" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C98" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D98" s="1">
         <v>45689</v>
@@ -2631,13 +2631,13 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>181</v>
+      </c>
+      <c r="B99" t="s">
+        <v>182</v>
+      </c>
+      <c r="C99" t="s">
         <v>183</v>
-      </c>
-      <c r="B99" t="s">
-        <v>184</v>
-      </c>
-      <c r="C99" t="s">
-        <v>185</v>
       </c>
       <c r="D99" s="1">
         <v>45658</v>
@@ -2648,13 +2648,13 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B100" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C100" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D100" s="1">
         <v>45839</v>
@@ -2662,13 +2662,13 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B101" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C101" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D101" s="1">
         <v>45901</v>
@@ -2676,13 +2676,13 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B102" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C102" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D102" s="1">
         <v>46082</v>
@@ -2691,13 +2691,13 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B103" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C103" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D103" s="1">
         <v>46082</v>
@@ -2706,13 +2706,13 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B104" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C104" t="s">
-        <v>19</v>
+        <v>197</v>
       </c>
       <c r="D104" s="1">
         <v>45901</v>
@@ -2721,13 +2721,13 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B105" t="s">
+        <v>195</v>
+      </c>
+      <c r="C105" t="s">
         <v>197</v>
-      </c>
-      <c r="C105" t="s">
-        <v>19</v>
       </c>
       <c r="D105" s="1">
         <v>45901</v>
@@ -2741,10 +2741,10 @@
         <v>5</v>
       </c>
       <c r="B106" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C106" t="s">
-        <v>19</v>
+        <v>197</v>
       </c>
       <c r="D106" s="1">
         <v>46082</v>
@@ -2753,13 +2753,13 @@
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B107" t="s">
+        <v>195</v>
+      </c>
+      <c r="C107" t="s">
         <v>197</v>
-      </c>
-      <c r="C107" t="s">
-        <v>19</v>
       </c>
       <c r="D107" s="1">
         <v>45170</v>
@@ -2789,15 +2789,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="5d5a2885-0f9b-4d04-9bc1-f867a2376b8a">
@@ -2806,6 +2797,15 @@
     <TaxCatchAll xmlns="6cbc0c5a-d948-46e5-8624-1bad210f77c7" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3058,20 +3058,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{052A151B-9EBC-4A5B-80E8-331BB541A51E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FDD2033D-62C9-49C5-95D2-9D0E2397323D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="5d5a2885-0f9b-4d04-9bc1-f867a2376b8a"/>
     <ds:schemaRef ds:uri="6cbc0c5a-d948-46e5-8624-1bad210f77c7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{052A151B-9EBC-4A5B-80E8-331BB541A51E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>